<commit_message>
refactor: rename company from NovaCommerce to Corporativo JUC (centralized in config.py)
</commit_message>
<xml_diff>
--- a/data/raw/sheets/promociones.xlsx
+++ b/data/raw/sheets/promociones.xlsx
@@ -522,7 +522,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Aniversario NovaCommerce</t>
+          <t>Aniversario Corporativo JUC</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -774,7 +774,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Aniversario NovaCommerce</t>
+          <t>Aniversario Corporativo JUC</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -802,7 +802,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Aniversario NovaCommerce</t>
+          <t>Aniversario Corporativo JUC</t>
         </is>
       </c>
       <c r="C14" t="n">

</xml_diff>